<commit_message>
Night Sky off, and a few more changes
</commit_message>
<xml_diff>
--- a/display/EcoGainsSim_HC_v4.xlsx
+++ b/display/EcoGainsSim_HC_v4.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Y188"/>
+  <dimension ref="B2:Y190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.75" customWidth="1" min="1" max="1"/>
@@ -5768,7 +5768,7 @@
     <row r="183">
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Night Sky: SIMULATED column = bottom-up FULL-ROLLOUT value (ladder x daily-max-streak survival x active days). CURRENT is A/B-diluted, so the diff mixes rollout effect with dilution.</t>
+          <t>Night Sky: CARRIED by default (NS_SIMULATE = false in EcoGainsSim_v4.gs - the bottom-up model overestimates actual NS gains; open question). Flag true -&gt; full-rollout sim (segment ladder x survival over data_streaks max-streak p25-p90 x 1.25 effective-streak factor x active days); CURRENT is A/B-diluted, so DIFF would read as ROLLOUT EFFECT.</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,21 @@
     <row r="188">
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>After editing a calendar: menu EcoGainsSim ▸ Precompute calendars (writes hidden cal_parsed; engine prefers it). Sanity canary: the Kite Festival row must SHRINK vs measured (D≈0.34 @0-9). If every event row equals measured, the calendar read failed.</t>
+          <t>Reward-config edits FLOW (since 2026-07-06): editing rewards or requirements on any _v2 sheet reprices its row (R = v2/base ladder at the measured rank / progress distribution). Base sheets = the measured world; leave them untouched. TaD milestone rewards are the exception (base pays 0 -&gt; no anchor -&gt; carried).</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>Kite Festival is priced as a LEADERBOARD (since 2026-07-06): payouts are zero-sum per league of 60, so duration does not move them; D=1 and the row GROWS ~x1.3 via cadence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>After editing a calendar: menu EcoGainsSim ▸ Precompute calendars (writes hidden cal_parsed; engine prefers it). Sanity canary: the Kite Festival row must GROW ~x1.3 vs measured. If every event row equals measured, the calendar read failed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
engine: refresh-nonce model - sim_refresh!A1 argument instead of clear/re-set formulas
refreshSims_ now bumps a timestamp nonce in sim_refresh!A1 that every sim formula carries as an
ignored trailing argument - Google re-runs on argument change, nothing is ever cleared, so the
periodic disappearing-formula failure (onEdit 30s hard-kill mid clear->restore) is gone.
refreshSims_ also self-heals: appends the nonce to bare formulas, repairs #REF! decay, restores
missing anchors from a document-properties snapshot. CalStats E38 takes the nonce too.
_build_hc_v4 writes nonce-carrying anchors; restored/ exports regenerated; _nonce_test.js covers
the plumbing. Rides along in v4: REFRESH_WATCH gains data_econ + data_econ_daily (NET inputs;
data_econ still needs menu > Fill Sim per Segment after edits).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/display/EcoGainsSim_HC_v4.xlsx
+++ b/display/EcoGainsSim_HC_v4.xlsx
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="C8" s="10">
-        <f>LET(payer, $C$3, segment, $B$6, ECOGAINS_SIM(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$6, ECOGAINS_SIM(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="D8" s="10" t="n"/>
@@ -716,7 +716,7 @@
       <c r="L8" s="10" t="n"/>
       <c r="M8" s="10" t="n"/>
       <c r="O8" s="11">
-        <f>LET(payer, $C$3, segment, $B$6, ECOGAINS_DIFF(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$6, ECOGAINS_DIFF(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="P8" s="11" t="n"/>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="C37" s="10">
-        <f>LET(payer, $C$3, segment, $B$35, ECOGAINS_SIM(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$35, ECOGAINS_SIM(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="D37" s="10" t="n"/>
@@ -1581,7 +1581,7 @@
       <c r="L37" s="10" t="n"/>
       <c r="M37" s="10" t="n"/>
       <c r="O37" s="11">
-        <f>LET(payer, $C$3, segment, $B$35, ECOGAINS_DIFF(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$35, ECOGAINS_DIFF(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="P37" s="11" t="n"/>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="C66" s="10">
-        <f>LET(payer, $C$3, segment, $B$64, ECOGAINS_SIM(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$64, ECOGAINS_SIM(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="D66" s="10" t="n"/>
@@ -2446,7 +2446,7 @@
       <c r="L66" s="10" t="n"/>
       <c r="M66" s="10" t="n"/>
       <c r="O66" s="11">
-        <f>LET(payer, $C$3, segment, $B$64, ECOGAINS_DIFF(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$64, ECOGAINS_DIFF(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="P66" s="11" t="n"/>
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="C95" s="10">
-        <f>LET(payer, $C$3, segment, $B$93, ECOGAINS_SIM(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$93, ECOGAINS_SIM(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="D95" s="10" t="n"/>
@@ -3311,7 +3311,7 @@
       <c r="L95" s="10" t="n"/>
       <c r="M95" s="10" t="n"/>
       <c r="O95" s="11">
-        <f>LET(payer, $C$3, segment, $B$93, ECOGAINS_DIFF(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$93, ECOGAINS_DIFF(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="P95" s="11" t="n"/>
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="C124" s="10">
-        <f>LET(payer, $C$3, segment, $B$122, ECOGAINS_SIM(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$122, ECOGAINS_SIM(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="D124" s="10" t="n"/>
@@ -4176,7 +4176,7 @@
       <c r="L124" s="10" t="n"/>
       <c r="M124" s="10" t="n"/>
       <c r="O124" s="11">
-        <f>LET(payer, $C$3, segment, $B$122, ECOGAINS_DIFF(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$122, ECOGAINS_DIFF(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="P124" s="11" t="n"/>
@@ -5027,7 +5027,7 @@
         </is>
       </c>
       <c r="C153" s="10">
-        <f>LET(payer, $C$3, segment, $B$151, ECOGAINS_SIM(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$151, ECOGAINS_SIM(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="D153" s="10" t="n"/>
@@ -5041,7 +5041,7 @@
       <c r="L153" s="10" t="n"/>
       <c r="M153" s="10" t="n"/>
       <c r="O153" s="11">
-        <f>LET(payer, $C$3, segment, $B$151, ECOGAINS_DIFF(payer, segment))</f>
+        <f>LET(payer, $C$3, segment, $B$151, ECOGAINS_DIFF(payer, segment, sim_refresh!$A$1))</f>
         <v/>
       </c>
       <c r="P153" s="11" t="n"/>

</xml_diff>